<commit_message>
Fix dividend timing and partial-history returns
</commit_message>
<xml_diff>
--- a/templates/generic_transactions_template.xlsx
+++ b/templates/generic_transactions_template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transactions'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transactions'!$A$1:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -506,17 +506,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,35 +530,50 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Ex Date</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Start</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Coverage End</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Price Per Share</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Fees</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -565,19 +583,26 @@
       <c r="A2" s="3" t="n">
         <v>46036</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>DEPOSIT</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n">
         <v>5000</v>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Transfer from checking</t>
         </is>
@@ -587,27 +612,34 @@
       <c r="A3" s="3" t="n">
         <v>46037</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>SCHD</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="G3" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="H3" s="6" t="n">
         <v>27.5</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Initial purchase</t>
         </is>
@@ -617,23 +649,32 @@
       <c r="A4" s="3" t="n">
         <v>46056</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="n">
+        <v>46052</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>DIVIDEND</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>SCHD</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n">
         <v>8.25</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Cash dividend received</t>
         </is>
@@ -643,27 +684,34 @@
       <c r="A5" s="3" t="n">
         <v>46056</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>DRIP</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>SCHD</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.3</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="H5" s="6" t="n">
         <v>27.5</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Dividend reinvestment shares</t>
         </is>
@@ -673,23 +721,30 @@
       <c r="A6" s="3" t="n">
         <v>46073</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>TRANSFER IN</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>JEPI</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="G6" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Shares moved from another broker</t>
         </is>
@@ -699,27 +754,34 @@
       <c r="A7" s="3" t="n">
         <v>46091</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>SCHD</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="G7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="H7" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Partial sale</t>
         </is>
@@ -729,28 +791,35 @@
       <c r="A8" s="3" t="n">
         <v>46093</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>WITHDRAWAL</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n">
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Transfer to checking</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:K8"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid transaction type" error="Choose BUY, SELL, DIVIDEND, DRIP, DEPOSIT, WITHDRAWAL, TRANSFER IN, TRANSFER OUT, FEE, or INTEREST." promptTitle="Transaction type" prompt="Select the kind of transaction." type="list">
+    <dataValidation sqref="E2:E1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid transaction type" error="Choose BUY, SELL, DIVIDEND, DRIP, DEPOSIT, WITHDRAWAL, TRANSFER IN, TRANSFER OUT, FEE, or INTEREST." promptTitle="Transaction type" prompt="Select the kind of transaction." type="list">
       <formula1>"BUY,SELL,DIVIDEND,DRIP,DEPOSIT,WITHDRAWAL,TRANSFER IN,TRANSFER OUT,FEE,INTEREST"</formula1>
     </dataValidation>
   </dataValidations>
@@ -764,7 +833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -834,166 +903,232 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Ex Date</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Dividends (recommended)</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Determines how the row affects holdings, income, and account cash flows.</t>
+          <t>Ex-dividend date used for investment-performance timing; cash totals still use Date.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>BUY, SELL, DIVIDEND, DRIP, DEPOSIT, WITHDRAWAL, TRANSFER IN, TRANSFER OUT, FEE, or INTEREST</t>
+          <t>2026-01-30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Ticker</t>
+          <t>Coverage Start</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Securities only</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Security ticker, trimmed and uppercased. Leave blank for DEPOSIT, WITHDRAWAL, FEE, and INTEREST.</t>
+          <t>First date for which this file contains complete broker activity and distributions.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>SCHD</t>
+          <t>2026-01-01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Shares</t>
+          <t>Coverage End</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Trades and transfers</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Positive share quantity for BUY, SELL, DRIP, TRANSFER IN, and TRANSFER OUT.</t>
+          <t>Last date for which this file contains complete broker activity and distributions.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>10 or 0.3250</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Price Per Share</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Trades only</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Execution price for BUY, SELL, and DRIP. Optional for transfers; blank values them at that day's close.</t>
+          <t>Determines how the row affects holdings, income, and account cash flows.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>27.50</t>
+          <t>BUY, SELL, DIVIDEND, DRIP, DEPOSIT, WITHDRAWAL, TRANSFER IN, TRANSFER OUT, FEE, or INTEREST</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Fees</t>
+          <t>Ticker</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Securities only</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Commission or transaction fee; blank defaults to zero.</t>
+          <t>Security ticker, trimmed and uppercased. Leave blank for DEPOSIT, WITHDRAWAL, FEE, and INTEREST.</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>SCHD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Shares</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Cash rows</t>
+          <t>Trades and transfers</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Total cash for DIVIDEND, DEPOSIT, WITHDRAWAL, FEE, and INTEREST rows. Enter it as a positive number; the type decides whether money came in or went out (INTEREST keeps its sign, so margin interest charged can be negative).</t>
+          <t>Positive share quantity for BUY, SELL, DRIP, TRANSFER IN, and TRANSFER OUT.</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>8.25 or 5000</t>
+          <t>10 or 0.3250</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Price Per Share</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Trades only</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Execution price for BUY, SELL, and DRIP. Optional for transfers; blank values them at that day's close.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>27.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Commission or transaction fee; blank defaults to zero.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Cash rows</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Total cash for DIVIDEND, DEPOSIT, WITHDRAWAL, FEE, and INTEREST rows. Enter it as a positive number; the type decides whether money came in or went out (INTEREST keeps its sign, so margin interest charged can be negative).</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>8.25 or 5000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Optional description saved with the transaction.</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Initial purchase</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>BUY, SELL, and DRIP rows update positions when the transaction ledger is the portfolio's source of truth. If current holdings already exist, the import keeps those share counts and adds the transactions for history, cost-basis support, dividend tracking, and realized gains—matching broker transaction imports.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="72" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Account Alpha on the Dashboard: DEPOSIT, WITHDRAWAL, TRANSFER IN, and TRANSFER OUT rows let the app separate money you added or took out from what the account earned. When a file contains any of these rows, the app treats the file's first-to-last date as a complete record of money in and out, so include every deposit and withdrawal for that stretch. A period with no money movements can be marked complete on the Holdings screen under Deposits &amp; Withdrawals.</t>
         </is>
@@ -1002,9 +1137,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A18:D18"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>